<commit_message>
Exact all-keywords bulk: fixed bidding instead of down-only
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJUn53DicDcqHAh1hw7jdv
</commit_message>
<xml_diff>
--- a/deliverables/coolinens-launch/bulk/COOLINENS_Cooling_Pillowcases_Exact_All_Keywords_Bulk_20261004.xlsx
+++ b/deliverables/coolinens-launch/bulk/COOLINENS_Cooling_Pillowcases_Exact_All_Keywords_Bulk_20261004.xlsx
@@ -747,7 +747,7 @@
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>Dynamic bids - down only</t>
+          <t>Fixed bid</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
       </c>
       <c r="AG7" t="inlineStr">
         <is>
-          <t>Dynamic bids - down only</t>
+          <t>Fixed bid</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="AG12" t="inlineStr">
         <is>
-          <t>Dynamic bids - down only</t>
+          <t>Fixed bid</t>
         </is>
       </c>
     </row>
@@ -1362,7 +1362,7 @@
       </c>
       <c r="AG16" t="inlineStr">
         <is>
-          <t>Dynamic bids - down only</t>
+          <t>Fixed bid</t>
         </is>
       </c>
     </row>
@@ -1541,7 +1541,7 @@
       </c>
       <c r="AG20" t="inlineStr">
         <is>
-          <t>Dynamic bids - down only</t>
+          <t>Fixed bid</t>
         </is>
       </c>
     </row>
@@ -1759,7 +1759,7 @@
       </c>
       <c r="AG25" t="inlineStr">
         <is>
-          <t>Dynamic bids - down only</t>
+          <t>Fixed bid</t>
         </is>
       </c>
     </row>
@@ -1977,7 +1977,7 @@
       </c>
       <c r="AG30" t="inlineStr">
         <is>
-          <t>Dynamic bids - down only</t>
+          <t>Fixed bid</t>
         </is>
       </c>
     </row>
@@ -2195,7 +2195,7 @@
       </c>
       <c r="AG35" t="inlineStr">
         <is>
-          <t>Dynamic bids - down only</t>
+          <t>Fixed bid</t>
         </is>
       </c>
     </row>
@@ -2413,7 +2413,7 @@
       </c>
       <c r="AG40" t="inlineStr">
         <is>
-          <t>Dynamic bids - down only</t>
+          <t>Fixed bid</t>
         </is>
       </c>
     </row>
@@ -2631,7 +2631,7 @@
       </c>
       <c r="AG45" t="inlineStr">
         <is>
-          <t>Dynamic bids - down only</t>
+          <t>Fixed bid</t>
         </is>
       </c>
     </row>
@@ -2849,7 +2849,7 @@
       </c>
       <c r="AG50" t="inlineStr">
         <is>
-          <t>Dynamic bids - down only</t>
+          <t>Fixed bid</t>
         </is>
       </c>
     </row>
@@ -3067,7 +3067,7 @@
       </c>
       <c r="AG55" t="inlineStr">
         <is>
-          <t>Dynamic bids - down only</t>
+          <t>Fixed bid</t>
         </is>
       </c>
     </row>
@@ -3285,7 +3285,7 @@
       </c>
       <c r="AG60" t="inlineStr">
         <is>
-          <t>Dynamic bids - down only</t>
+          <t>Fixed bid</t>
         </is>
       </c>
     </row>
@@ -3699,7 +3699,7 @@
       </c>
       <c r="AG69" t="inlineStr">
         <is>
-          <t>Dynamic bids - down only</t>
+          <t>Fixed bid</t>
         </is>
       </c>
     </row>
@@ -4113,7 +4113,7 @@
       </c>
       <c r="AG78" t="inlineStr">
         <is>
-          <t>Dynamic bids - down only</t>
+          <t>Fixed bid</t>
         </is>
       </c>
     </row>
@@ -4621,7 +4621,7 @@
       </c>
       <c r="AG89" t="inlineStr">
         <is>
-          <t>Dynamic bids - down only</t>
+          <t>Fixed bid</t>
         </is>
       </c>
     </row>
@@ -4894,7 +4894,7 @@
       </c>
       <c r="AG95" t="inlineStr">
         <is>
-          <t>Dynamic bids - down only</t>
+          <t>Fixed bid</t>
         </is>
       </c>
     </row>
@@ -5214,7 +5214,7 @@
       </c>
       <c r="AG102" t="inlineStr">
         <is>
-          <t>Dynamic bids - down only</t>
+          <t>Fixed bid</t>
         </is>
       </c>
     </row>
@@ -5581,7 +5581,7 @@
       </c>
       <c r="AG110" t="inlineStr">
         <is>
-          <t>Dynamic bids - down only</t>
+          <t>Fixed bid</t>
         </is>
       </c>
     </row>
@@ -5807,7 +5807,7 @@
       </c>
       <c r="AG115" t="inlineStr">
         <is>
-          <t>Dynamic bids - down only</t>
+          <t>Fixed bid</t>
         </is>
       </c>
     </row>
@@ -6080,7 +6080,7 @@
       </c>
       <c r="AG121" t="inlineStr">
         <is>
-          <t>Dynamic bids - down only</t>
+          <t>Fixed bid</t>
         </is>
       </c>
     </row>
@@ -6400,7 +6400,7 @@
       </c>
       <c r="AG128" t="inlineStr">
         <is>
-          <t>Dynamic bids - down only</t>
+          <t>Fixed bid</t>
         </is>
       </c>
     </row>
@@ -6767,7 +6767,7 @@
       </c>
       <c r="AG136" t="inlineStr">
         <is>
-          <t>Dynamic bids - down only</t>
+          <t>Fixed bid</t>
         </is>
       </c>
     </row>

</xml_diff>